<commit_message>
Automation Selenium Sprint-Evaluation Day
</commit_message>
<xml_diff>
--- a/NoBroker/NoBroker/src/test/resource/ExcelData/Data.xlsx
+++ b/NoBroker/NoBroker/src/test/resource/ExcelData/Data.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28730"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{C8C14D6E-BB67-46EF-BD7C-9C2DE5752D53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{F5185905-5246-403E-847A-90B9F13D95BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -13,7 +13,7 @@
     <sheet name="PhoneNumber" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="0"/>
-  <oleSize ref="A1:G14"/>
+  <oleSize ref="A1:N15"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>

</xml_diff>